<commit_message>
confeccion de tablas de resultados
</commit_message>
<xml_diff>
--- a/resultados/resultados_RS_cv_vs_test_predict-faults_sofo_f1-macro.xlsx
+++ b/resultados/resultados_RS_cv_vs_test_predict-faults_sofo_f1-macro.xlsx
@@ -498,7 +498,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -609,7 +608,7 @@
         <v>0.98299999999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>18</v>
       </c>
@@ -657,7 +656,7 @@
         <v>0.98299999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>18</v>
       </c>
@@ -705,7 +704,7 @@
         <v>0.98099999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>22</v>
       </c>
@@ -761,7 +760,7 @@
         <v>0.98099999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>22</v>
       </c>
@@ -817,7 +816,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="7" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>21</v>
       </c>
@@ -923,7 +922,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="9" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
@@ -979,7 +978,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="10" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>20</v>
       </c>
@@ -1029,7 +1028,7 @@
         <v>0.97599999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>21</v>
       </c>
@@ -1129,7 +1128,7 @@
         <v>0.97699999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>20</v>
       </c>
@@ -1235,7 +1234,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -1285,7 +1284,7 @@
         <v>0.97299999999999998</v>
       </c>
     </row>
-    <row r="16" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>19</v>
       </c>
@@ -1437,11 +1436,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:R18">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="0"/>
-      </filters>
-    </filterColumn>
     <sortState ref="A2:R18">
       <sortCondition descending="1" ref="Q1:Q18"/>
     </sortState>

</xml_diff>